<commit_message>
test(e2e): tabela de endpoints por RF, evidências, cobertura JaCoCo e planilhas das etapas 12 e 13
- docs/testes: 452 passos / 368 endpoints com status esperado; por passo: RF (Trello), CA,
  endpoint, status, tabelas gravadas no MySQL (general_log) e tela que relê o dado
- cobertura medida com o agente JaCoCo durante o teste: 74,4% das linhas do backend
- docs/planilhas: IA por RF/RNF e entidades/bancos por RF/RNF (RF1-RF39), gerados do código
- guia de rubricas atualizado (RF25-RF39, E2E, cobertura, estado real de cada critério)
- scripts/e2e e scripts/diagramas no repositório, com caminhos configuráveis
- barra lateral dentro de um container de fundo branco (desktop, gaveta e barra inferior)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F9izb54cwzjj9BQQabn6GG
</commit_message>
<xml_diff>
--- a/docs/rubricas/GUIA_RUBRICAS.xlsx
+++ b/docs/rubricas/GUIA_RUBRICAS.xlsx
@@ -43,17 +43,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -64,6 +59,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F1F1F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,7 +86,7 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -99,7 +99,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,22 +533,22 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Serviços de aplicação para RF1–RF36 e RNF1–RNF12 em fai-application/.../service; entidades e migrações V1–V6; docs/novo-projeto/tabela-*.md.</t>
+          <t>39 RFs do Trello (RF1–RF39) com endpoint e tela; 368 endpoints REST no inventário; teste ponta a ponta com 452 passos cobrindo todos os endpoints (docs/testes/TABELA_ENDPOINTS_POR_RF.md/.xlsx: RF, CA, endpoint, status, banco em que salvou, tela que exibe). Planilhas da etapa 12 (docs/planilhas/) servem de checklist RF a RF.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Bloco 8 (API REST de todos os serviços) e bloco 11 (frontend com todas as telas).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Levar aos professores a lista de RFs do escopo acordado e marcar, RF a RF, onde está a tela e o endpoint (a planilha de IA/entidades do bloco 12 serve de checklist).</t>
+          <t>Levar aos professores a lista de RFs do escopo acordado e a tabela de endpoints por RF; confirmar se RF33–RF39 (Passarela 3D, Eras, Coleções, Foto com manequim, FLAIR, Cupons, Criar guarda-roupa 3D) entram no escopo.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Board do Trello com HUs/RFs; HUs e critérios de aceite em markdowns/HU*.md e markdowns/02-rf-reestruturados-e-criterios-aceite.md.</t>
+          <t>Board do Trello com RF1–RF39 (critérios de aceite nos cards); HUs e CAs em markdowns/; histórico de commits por RF.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -601,24 +601,24 @@
           <t>Frontend bem acabado, mensagens informativas e resiliente a erros</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Backend já devolve erros de negócio com código e mensagem (ApiException, ex.: 409 PECA_INDISPONIVEL, 429 cota de IA, 422 validação); tipografia oficial (lib/design/typography.css) e 77 ícones FAI.</t>
+          <t>Next.js com toasts de sucesso/erro (useToast), EmptyState, ErrorState com 'tentar de novo', Skeleton de carregamento, mensagens de negócio vindas da API (409/422/429), aviso de fallback de IA (motor local) e status por fonte no buscador de marcas; capturas em docs/novos-rf/telas-*/.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bloco 11: toasts de sucesso/erro, estados vazios, skeletons de carregamento, error boundary por página, retry em falha de rede, mensagens de fallback de IA.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Na demo, provocar um erro de propósito (ex.: sem internet, campo inválido) e mostrar a mensagem.</t>
+          <t>Na demo, provocar um erro de propósito (campo inválido, peça indisponível no look) e mostrar a mensagem.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -638,17 +638,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Casos de uso prontos e compilando; DTOs/records em JSON; módulo fai-web.</t>
+          <t>368 endpoints REST (fai-web/.../controller) com verbos e códigos HTTP (200/201/202/204/400/403/404/409/422/429), GlobalExceptionHandler com JSON de erro (code, message, details, correlationId), springdoc-openapi + Swagger UI.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Bloco 8: controllers REST (substantivos no plural, verbos HTTP, 201/204/404/409/422), GlobalExceptionHandler com application/problem+json, OpenAPI.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -671,24 +671,24 @@
           <t>Dados relevantes persistidos em banco</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>MySQL via Flyway V1–V6 (JPA, UUID CHAR(36), campos sensíveis cifrados com AES-GCM); auditoria em audit_log; log de inferência de IA; Cassandra (timeline) e Redis (contadores/cache).</t>
+          <t>MySQL com Flyway V1–V21 (79 entidades JPA; campos sensíveis cifrados com AES-GCM); audit_log; ai_inference_log; prova por endpoint do que foi gravado (general_log do MySQL) em docs/testes/; projeções Redis/Cassandra/OpenSearch e mídia em S3 atrás de feature flags (docs/planilhas/Entidades_BD_por_RF_RNF.xlsx).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Bloco 10: subir a aplicação contra o MySQL e validar ponta a ponta.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Levar o diagrama ER (docs/novo-projeto/tabela-entidades-rf-bancos.md + markdowns/uml-casos-er-classes.md).</t>
+          <t>Levar o diagrama de classes v4 (docs/diagramas/fashionai-classes-v4.puml) e a planilha de entidades por RF.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -708,17 +708,17 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Perfis PESSOAL, MARCA e CELEBRIDADE (ProfileType) + papel USER/ADMIN (User.role); guard.requireAdmin em AdminService/ChallengeService/BackgroundStudioService; dashboard de emissor só para MARCA/CELEBRIDADE; ResourceOwnerAuthorizationTest.</t>
+          <t>Perfis PESSOAL, MARCA e CELEBRIDADE + papel ADMIN; guard.requireAdmin/requireOwner no backend (403 ACESSO_NEGADO testado no E2E, ex.: usuário comum no criador de guarda-roupa RF39 e no admin); menus e rotas por perfil no frontend (aba Criar guarda-roupa 3D só para MARCA/CELEBRIDADE; /admin só para ADMIN); ResourceOwnerAuthorizationTest.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Bloco 8: @PreAuthorize/filtros por papel e 403 JSON. Bloco 11: guarda de rota e menus ocultos por perfil.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -743,17 +743,17 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>DashboardService (admin e emissor), filtros período/país/tipo de perfil, alertas, layout de widgets salvo por usuário; V6 com procedures sp_admin_kpis/sp_timeseries, views vw_country_insights/vw_brand_usage e índices.</t>
+          <t>/admin/dashboard e dashboard do emissor (marca/celebridade) com filtros período/país/tipo de perfil, gráficos e widgets salvos por usuário; procedures sp_admin_kpis/sp_timeseries e views (V6); endpoints testados no E2E.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Bloco 8 (endpoint /api/admin/dashboard) e bloco 11 (gráficos de linha/barra/pizza/mapa).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -776,14 +776,14 @@
           <t>Git organizado (branches, commits) com participação de TODOS os alunos</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>RISCO</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Branches por feature e PRs (#8, #12); commits no padrão Conventional Commits (feat/fix/chore com RF no escopo). ATENÇÃO: `git shortlog -sn --all` neste repositório mostra commits só de Matheus + bots; nenhum do Bryan.</t>
+          <t>Branch por frente e commits no padrão Conventional Commits com o RF no escopo. ATENÇÃO: `git shortlog -sn --all` mostrava em 24/09 Matheus (82), Claude (42) e copilot (10); nenhum commit do Bryan.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Bryan precisa commitar com a própria conta (docs das sprints, testes, telas, revisões de PR). Todo PR revisado/aprovado pelo outro integrante. Apresentar também o histórico do repositório SAI-TCC-2026. Confirmar com os professores a política sobre commits assistidos por IA (co-autoria aparece no log).</t>
+          <t>Bryan precisa commitar com a própria conta (docs das sprints, testes, telas, revisões de PR). Todo PR revisado/aprovado pelo outro integrante. Confirmar com os professores a política sobre commits assistidos por IA (a co-autoria aparece no log).</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -901,14 +901,14 @@
       <c r="F2" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>a) GROUP BY no MysqlAnalyticsAdapter (uso de IA, marcas, países, faixas de Hype/Inventory, funil de selos); b) índices UNIQUE que impõem regras (username/e-mail únicos, seguir 1×, 1 Look do Dia por dia, 1 reação por alvo, 1 voto por entrada de desafio, ledger idempotente de FAI Points) + índices de V6; c) procedures sp_admin_kpis, sp_timeseries, sp_purge_notifications e views.</t>
+          <t>a) GROUP BY no MysqlAnalyticsAdapter (uso de IA, marcas, países, faixas de Hype/Inventory, funil de selos); b) índices UNIQUE que impõem regras (username/e-mail únicos, seguir 1×, 1 Look do Dia por dia, 1 reação por alvo, 1 voto por entrada de desafio, ledger idempotente de FAI Points); c) procedures sp_admin_kpis, sp_timeseries, sp_purge_notifications e views; EXPLAIN em docs/banco/EXPLAIN_DASHBOARD.md.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -944,19 +944,19 @@
       <c r="F3" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Hospedagem Vercel; storage S3/Vercel Blob (fotos e cards); IA generativa (Claude, Gemini, FASHN, Meshy); e-mail transacional Resend; login federado Google; MySQL gerenciado.</t>
+          <t>Adaptadores prontos: S3 (mídia), Claude/Gemini/FASHN/Meshy/Photoroom (IA), Resend (e-mail), Open-Meteo (clima), Wikidata/GitHub (buscador de marcas); frontend na Vercel. Neste ambiente só o GitHub é alcançável (rede restrita) e não há chaves de IA: tudo roda no fallback local.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Bloco 9 (adaptadores) + deploy; no TDE, justificar cada serviço pelo problema de negócio.</t>
+          <t>Deploy com as chaves reais; no TDE, justificar cada serviço pelo problema de negócio e mostrar 1 chamada real de cada.</t>
         </is>
       </c>
     </row>
@@ -989,17 +989,17 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Layout de widgets do dashboard salvo por usuário (user_preferences.dashboard_layout_json); Background Studio/skins de cards; tokens de tipografia.</t>
+          <t>Temas claro/escuro/alto contraste (data-theme), cor do container e fundo da interface salvos em user_preferences, widgets do dashboard salvos por usuário, Background Studio/skins de cards, layout mobile com menu recolhível.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Bloco 11: temas claro/escuro/alto contraste, breakpoints mobile, arrastar/ocultar widgets com salvamento.</t>
+          <t>Na demo, trocar o tema e mostrar a tela no celular.</t>
         </is>
       </c>
     </row>
@@ -1032,17 +1032,17 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>HU01–HU20 com critérios de aceite, casos de uso e ER (markdowns/uml-*.md), diagramas de atividade (markdowns/05-diagramas-atividade.md, RF33_Vista-me_Atividades.puml), diagramas de sequência dos pipelines RF4/RF18.</t>
+          <t>Pacote de diagramas 13 (atividades, sequência, estados, classes e componentes de RF1–RF39; RF25–RF39 gerados do código; RF4 v3 e RF5 v4 com o buscador de marcas); CAs por RF nos cards do Trello.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Marcar em cada sprint do TDE qual HU/diagrama modelou os cards daquela sprint.</t>
+          <t>Marcar em cada sprint do TDE qual diagrama modelou os cards daquela sprint.</t>
         </is>
       </c>
     </row>
@@ -1073,19 +1073,19 @@
       <c r="F6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>springdoc-openapi com @Operation (RF/CA no sumário) em todos os endpoints; README; payloads reais de cada endpoint nos cartões de evidência do teste ponta a ponta (docs/testes/).</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Bloco 8: springdoc-openapi com @Operation/@ExampleObject por endpoint; README.md (o que é, como subir, como rodar).</t>
+          <t>Mostrar o Swagger UI e um cartão de evidência (requisição → resposta → SQL).</t>
         </is>
       </c>
     </row>
@@ -1116,19 +1116,19 @@
       <c r="F7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Flyway V1–V6 (baseline, RFs completos, seed de marcas, critérios, Meu Guarda-Roupa, dashboard). Hoje todas as migrações têm a mesma data de commit, o que só garante a faixa de 30%.</t>
+          <t>Flyway V1–V21, uma migração por mudança (ex.: V20 loja/criador do guarda-roupa, V21 marca da peça pela busca web). As migrações foram commitadas em 2 dias (23 e 24/09), o que só garante a faixa de 30%.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>A partir desta sprint, toda mudança de banco entra como V7, V8…, commitada na sprint em que foi feita; tabela 'migração × sprint' no TDE.</t>
+          <t>A partir desta sprint, toda mudança de banco entra como V22, V23…, commitada na sprint em que foi feita; tabela 'migração × sprint' no TDE.</t>
         </is>
       </c>
     </row>
@@ -1159,14 +1159,14 @@
       <c r="F8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Hexagonal em módulos Maven (domain/application/infrastructure/web/bootstrap), ports &amp; adapters, Strategy + Chain of Responsibility no AiEngine (provedor principal → fallback → local), Observer (DomainEvents), Repository, Circuit Breaker/Retry (resilience4j), Facade (DashboardService).</t>
+          <t>Hexagonal em módulos Maven (domain/application/infrastructure/web/bootstrap), ports &amp; adapters, Strategy + Chain of Responsibility no AiEngine (primário → alternativa → local) e no buscador de marcas (Wikidata → Simple Icons → IA), Pipeline (LogoFilter, Flat Lay, Estúdio), Observer (eventos AFTER_COMMIT), Repository, Circuit Breaker/Retry, Facade.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1202,14 +1202,14 @@
       <c r="F9" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Anatomias dos cards (docs/anatomias), pranchas de telas (markdowns/04-telas-artefatos-e-pranchas.md).</t>
+          <t>Anatomias dos cards (v17), anatomia do DNA (v4), telas capturadas por RF em docs/.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1245,19 +1245,19 @@
       <c r="F10" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Locale do usuário já existe nas preferências.</t>
+          <t>Dicionários PT-BR/EN/ES (lib/i18n) e seletor de idioma no topo; formatos de data/número por locale.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Bloco 11: PT-BR/EN/ES com arquivos de mensagens; Intl.DateTimeFormat/NumberFormat; preços com moeda da loja.</t>
+          <t>Completar a tradução das telas novas (RF25–RF39) e mostrar a troca de idioma na demo.</t>
         </is>
       </c>
     </row>
@@ -1288,19 +1288,19 @@
       <c r="F11" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nome da cor em texto em toda peça, tema de alto contraste, combobox do buscador de marcas navegável por teclado (role=combobox/listbox), rótulos ARIA nos controles.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Público sugerido: pessoas com daltonismo (moda depende de cor). Estratégias: nome da cor em texto em toda peça, alto contraste, foco visível/teclado, alt text gerado. Teste com 3 pessoas e registrar.</t>
+          <t>Teste com 3 pessoas daltônicas e registrar.</t>
         </is>
       </c>
     </row>
@@ -1331,14 +1331,14 @@
       <c r="F12" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Frontend já com deploys automáticos Preview/Production na Vercel e variáveis por ambiente.</t>
+          <t>Frontend com deploys automáticos Preview/Production na Vercel. Não há workflow do GitHub Actions no repositório.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1374,19 +1374,19 @@
       <c r="F13" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Actuator (health/metrics), audit_log, ai_inference_log com custo/latência, alertas no dashboard.</t>
+          <t>Actuator com health/info/metrics/prometheus expostos, audit_log, ai_inference_log com custo/latência, correlationId em todo erro, alertas no dashboard.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Expor /actuator/prometheus e um painel Grafana Cloud com 1 alerta (erro 5xx ou custo de IA).</t>
+          <t>Painel Grafana Cloud lendo /actuator/prometheus com 1 alerta (erro 5xx ou custo de IA).</t>
         </is>
       </c>
     </row>
@@ -1417,14 +1417,14 @@
       <c r="F14" s="2" t="n">
         <v>1.5</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Pipelines de IA generativa: flat lay (RF4), provador virtual 2D (RF18), modelo 3D (Meshy), mosaico RF11.</t>
+          <t>Pipelines de imagem e IA: flat lay e estúdio (RF4), filtro de nitidez de logos (RF4), provador 2D (RF18), modelo 3D (RF16), quarto 3D e guarda-roupa 3D em WebGL (RF27/RF39), FLAIR (RF37).</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1460,14 +1460,14 @@
       <c r="F15" s="2" t="n">
         <v>0.6</v>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Critérios de aceite por RF (CA01..) já servem de casos de teste.</t>
+          <t>Teste ponta a ponta por CA (452 passos, 368 endpoints) com a tabela RF × CA × endpoint × banco × tela e até 5 fotos de evidência por endpoint (docs/testes/); bugs achados e corrigidos registrados nos commits 'fix(...)'.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1503,19 +1503,19 @@
       <c r="F16" s="2" t="n">
         <v>0.6</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Serviços puros e testáveis (Hype, Inventory Score, RoomAddress, faixas de clima, cursor de busca).</t>
+          <t>JaCoCo medido com o agente no backend durante o teste ponta a ponta (452 passos, 368 endpoints): 74,4% das linhas e 47,9% dos ramos do backend; 75,2% das linhas do fai-application e 90,5% do fai-web (docs/testes/COBERTURA_E2E.md, relatório HTML no pacote de evidências). Só com testes unitários a cobertura é baixa (3% no fai-application).</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Bloco 10: JaCoCo no pom + testes unitários das regras de cálculo; relatório HTML como evidência.</t>
+          <t>Mostrar o relatório HTML e explicar como foi medido (agente JaCoCo + scripts/e2e/jacoco_report.jsh); se os professores exigirem cobertura só por testes unitários, escrever testes de serviço com H2/Testcontainers.</t>
         </is>
       </c>
     </row>
@@ -1546,19 +1546,19 @@
       <c r="F17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Camadas lib/api (client), lib/hooks (useApi), components/ui, components/&lt;área&gt;; Provider de i18n e de tema.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Bloco 11: camadas api/ (client), hooks/, components/, features/; Adapter para a API; Provider para tema/i18n.</t>
+          <t>Documentar as camadas e o padrão Adapter da API em docs/arquitetura.</t>
         </is>
       </c>
     </row>
@@ -1589,19 +1589,19 @@
       <c r="F18" s="2" t="n">
         <v>0.45</v>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Cassandra (timeline particionada por usuário) e Redis com TTL (cache, rate limit).</t>
+          <t>Cassandra (timeline_by_user e notifications_by_user com TTL de 90/30 dias) e Redis (contadores, rate limit) atrás de feature flags; desligados no ambiente de teste.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Só vale se sobrar tempo: TTL explícito nas tabelas do Cassandra + validação de schema do payload.</t>
+          <t>Só vale se sobrar tempo: subir Cassandra/Redis no docker-compose e mostrar a timeline particionada.</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Capturas automatizadas com Playwright (fluxos RF4/RF5/RF13/RF39), mas sem testes unitários de componentes.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1761,19 +1761,19 @@
       <c r="F22" s="2" t="n">
         <v>0.3</v>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>docker-compose.dev.yml com MySQL/Redis/Cassandra/OpenSearch/MinIO.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>docker-compose.dev.yml (bloco 9) conta como parcial; Terraform só se sobrar tempo.</t>
+          <t>Terraform só se sobrar tempo.</t>
         </is>
       </c>
     </row>

</xml_diff>